<commit_message>
docs: record the UBER end-to-end roll-out and update the example report
</commit_message>
<xml_diff>
--- a/docs/examples/UBER-2026-08-06-workbook.xlsx
+++ b/docs/examples/UBER-2026-08-06-workbook.xlsx
@@ -10196,7 +10196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E180"/>
+  <dimension ref="A1:E182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -14994,6 +14994,52 @@
       </c>
       <c r="E180" t="inlineStr"/>
     </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>X-18</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>exception</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>untraced number '20%' in section 3 (debate-1)</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>X-19</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>exception</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>untraced number '20%' (debate-1)</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: record the UBER v2 re-run with untraced figures dropped and refresh the example report
</commit_message>
<xml_diff>
--- a/docs/examples/UBER-2026-08-06-workbook.xlsx
+++ b/docs/examples/UBER-2026-08-06-workbook.xlsx
@@ -10196,7 +10196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E182"/>
+  <dimension ref="A1:E181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -15012,33 +15012,10 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>untraced number '20%' in section 3 (debate-1)</t>
+          <t>dropped sentence with untraced number '20%' in section 3 (debate-1)</t>
         </is>
       </c>
       <c r="E181" t="inlineStr"/>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>X-19</t>
-        </is>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>exception</t>
-        </is>
-      </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="D182" t="inlineStr">
-        <is>
-          <t>untraced number '20%' (debate-1)</t>
-        </is>
-      </c>
-      <c r="E182" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>